<commit_message>
Se suben datos de Asia
</commit_message>
<xml_diff>
--- a/storage/app/pdfs/blending_asia_components.xlsx
+++ b/storage/app/pdfs/blending_asia_components.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://faro90mx-my.sharepoint.com/personal/rfavela_hcx_mx/Documents/F90/Operacion/Proyectos/Proyectos en curso/US Grains 013 (Analisis Global)/Asia Africa/1. Informacion AsiaAfrica/2. Blending/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{C8AD3F2B-3DD6-0C4F-A3F6-C4486412BC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{704B9ECD-D009-7845-BB66-F2DB5B434493}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{C8AD3F2B-3DD6-0C4F-A3F6-C4486412BC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B48AAAD5-5CA5-4540-BAA1-E8C4D309E7EA}"/>
   <bookViews>
-    <workbookView xWindow="4900" yWindow="4340" windowWidth="23280" windowHeight="12480" tabRatio="853" activeTab="3" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
+    <workbookView xWindow="4900" yWindow="4340" windowWidth="23280" windowHeight="12480" tabRatio="853" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="7" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="42">
   <si>
     <t>Content</t>
   </si>
@@ -57,9 +57,6 @@
   </si>
   <si>
     <t>Malaysia</t>
-  </si>
-  <si>
-    <t>Nigeria</t>
   </si>
   <si>
     <t>South Korea</t>
@@ -866,7 +863,7 @@
   <sheetPr>
     <tabColor rgb="FF002F60"/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="80.83203125" style="6" bestFit="1" customWidth="1"/>
@@ -889,7 +886,7 @@
     </row>
     <row r="5" spans="1:1" ht="15.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14" customHeight="1" x14ac:dyDescent="0.15">
@@ -936,9 +933,7 @@
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A15" s="10" t="s">
-        <v>9</v>
-      </c>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A16" s="10"/>
@@ -999,9 +994,6 @@
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A35" s="10"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A36" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1010,11 +1002,10 @@
   <hyperlinks>
     <hyperlink ref="A9" location="Japan!A1" display="Japan" xr:uid="{52F41C02-FB17-40E8-9576-770EFBC6C47F}"/>
     <hyperlink ref="A10" location="Malaysia!A1" display="Malaysia" xr:uid="{6F0D300B-3674-44F3-860D-53DBFD4A4C07}"/>
-    <hyperlink ref="A11" location="Nigeria!A1" display="Nigeria" xr:uid="{84C30D8F-C4FA-4E9E-9E02-0CF531E6F6A7}"/>
-    <hyperlink ref="A12" location="'South Korea'!A1" display="South Korea" xr:uid="{652D061D-962D-4590-BBB9-43E1018ED83F}"/>
-    <hyperlink ref="A13" location="Taiwan!A1" display="Taiwan" xr:uid="{8CFC9BDF-65CB-434D-AF2C-C796AD422BEA}"/>
-    <hyperlink ref="A14" location="Thailand!A1" display="Thailand" xr:uid="{2F667091-2D0F-4D5F-8738-53AB376E7F72}"/>
-    <hyperlink ref="A15" location="Vietnam!A1" display="Vietnam" xr:uid="{4A147E18-6BA9-4E62-A7AB-14236C01CD13}"/>
+    <hyperlink ref="A11" location="'South Korea'!A1" display="South Korea" xr:uid="{652D061D-962D-4590-BBB9-43E1018ED83F}"/>
+    <hyperlink ref="A12" location="Taiwan!A1" display="Taiwan" xr:uid="{8CFC9BDF-65CB-434D-AF2C-C796AD422BEA}"/>
+    <hyperlink ref="A13" location="Thailand!A1" display="Thailand" xr:uid="{2F667091-2D0F-4D5F-8738-53AB376E7F72}"/>
+    <hyperlink ref="A14" location="Vietnam!A1" display="Vietnam" xr:uid="{4A147E18-6BA9-4E62-A7AB-14236C01CD13}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1058,7 +1049,7 @@
     <row r="4" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
       <c r="B4" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -1066,7 +1057,7 @@
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="I4" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
@@ -1076,48 +1067,48 @@
     </row>
     <row r="5" spans="1:22" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I5" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="K5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="M5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A6" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="23">
         <v>7.2876397246129085E-2</v>
@@ -1159,7 +1150,7 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A7" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="23">
         <v>0.52367301008557898</v>
@@ -1202,7 +1193,7 @@
     </row>
     <row r="8" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="23">
         <v>1.3640294836796941E-2</v>
@@ -1251,7 +1242,7 @@
     </row>
     <row r="9" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="23">
         <v>0</v>
@@ -1300,7 +1291,7 @@
     </row>
     <row r="10" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="23">
         <v>1.7459577391100083E-2</v>
@@ -1349,7 +1340,7 @@
     </row>
     <row r="11" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="23">
         <v>2.2715865006459786E-2</v>
@@ -1398,7 +1389,7 @@
     </row>
     <row r="12" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="23">
         <v>1.3640294836796941E-2</v>
@@ -1447,7 +1438,7 @@
     </row>
     <row r="13" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="23">
         <v>0</v>
@@ -1496,7 +1487,7 @@
     </row>
     <row r="14" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="23">
         <v>5.9914995070630563E-2</v>
@@ -1545,7 +1536,7 @@
     </row>
     <row r="15" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="23">
         <v>2.0801449626115336E-2</v>
@@ -1594,7 +1585,7 @@
     </row>
     <row r="16" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="23">
         <v>0.12495874099989678</v>
@@ -1642,7 +1633,7 @@
     </row>
     <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="23">
         <v>0.12495874099989678</v>
@@ -1689,7 +1680,7 @@
     </row>
     <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="23">
         <v>0</v>
@@ -1736,7 +1727,7 @@
     </row>
     <row r="19" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="23">
         <v>0</v>
@@ -1783,7 +1774,7 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A20" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="23">
         <v>0</v>
@@ -1824,7 +1815,7 @@
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A21" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="23">
         <v>0</v>
@@ -1865,7 +1856,7 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A22" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="23">
         <v>5.3606358708611981E-3</v>
@@ -1906,7 +1897,7 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A23" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="23">
         <v>0</v>
@@ -1947,7 +1938,7 @@
     </row>
     <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="26">
         <v>2.2233780546404009</v>
@@ -1995,7 +1986,7 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="28">
         <v>89.175451125506029</v>
@@ -2037,7 +2028,7 @@
     <row r="28" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -2045,7 +2036,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="I28" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="31"/>
       <c r="K28" s="31"/>
@@ -2055,48 +2046,48 @@
     </row>
     <row r="29" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="D29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="F29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="20" t="s">
+      <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="L29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="M29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="20" t="s">
+      <c r="N29" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N29" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A30" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="23">
         <v>7.7547975493354959E-2</v>
@@ -2137,7 +2128,7 @@
     </row>
     <row r="31" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="23">
         <v>0.29765376758219914</v>
@@ -2186,7 +2177,7 @@
     </row>
     <row r="32" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="23">
         <v>7.3956756590389056E-2</v>
@@ -2235,7 +2226,7 @@
     </row>
     <row r="33" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33" s="23">
         <v>5.6571060648877493E-2</v>
@@ -2284,7 +2275,7 @@
     </row>
     <row r="34" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="23">
         <v>4.101497659408164E-2</v>
@@ -2333,7 +2324,7 @@
     </row>
     <row r="35" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="23">
         <v>4.7998207978600042E-2</v>
@@ -2382,7 +2373,7 @@
     </row>
     <row r="36" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="23">
         <v>7.3920903236094273E-5</v>
@@ -2431,7 +2422,7 @@
     </row>
     <row r="37" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="23">
         <v>0</v>
@@ -2480,7 +2471,7 @@
     </row>
     <row r="38" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="23">
         <v>1.2225034347280737E-4</v>
@@ -2529,7 +2520,7 @@
     </row>
     <row r="39" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="23">
         <v>0.11091985163115278</v>
@@ -2578,7 +2569,7 @@
     </row>
     <row r="40" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="23">
         <v>2.7680313957369952E-2</v>
@@ -2627,7 +2618,7 @@
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="23">
         <v>4.245231004561275E-2</v>
@@ -2675,7 +2666,7 @@
     </row>
     <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="23">
         <v>7.9781537324359095E-2</v>
@@ -2723,7 +2714,7 @@
     </row>
     <row r="43" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="23">
         <v>0</v>
@@ -2771,7 +2762,7 @@
     </row>
     <row r="44" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="23">
         <v>0</v>
@@ -2819,7 +2810,7 @@
     </row>
     <row r="45" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A45" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="23">
         <v>0.11450791108387884</v>
@@ -2867,7 +2858,7 @@
     </row>
     <row r="46" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="23">
         <v>2.9719158368090807E-2</v>
@@ -2915,7 +2906,7 @@
     </row>
     <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="23">
         <v>0</v>
@@ -2963,7 +2954,7 @@
     </row>
     <row r="48" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A48" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="26">
         <v>2.4212259613369422</v>
@@ -3011,7 +3002,7 @@
     </row>
     <row r="49" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A49" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="28">
         <v>96.000082408251302</v>
@@ -3732,7 +3723,7 @@
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
       <c r="B4" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -3740,7 +3731,7 @@
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="I4" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
@@ -3750,48 +3741,48 @@
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I5" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="K5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="M5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="23">
         <v>0.11303859929283797</v>
@@ -3839,7 +3830,7 @@
     </row>
     <row r="7" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="23">
         <v>0.53626425908667286</v>
@@ -3887,7 +3878,7 @@
     </row>
     <row r="8" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="23">
         <v>0</v>
@@ -3935,7 +3926,7 @@
     </row>
     <row r="9" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="23">
         <v>0</v>
@@ -3983,7 +3974,7 @@
     </row>
     <row r="10" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="23">
         <v>0</v>
@@ -4031,7 +4022,7 @@
     </row>
     <row r="11" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="23">
         <v>2.9603901584342961E-2</v>
@@ -4079,7 +4070,7 @@
     </row>
     <row r="12" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="23">
         <v>4.5100460673113893E-2</v>
@@ -4127,7 +4118,7 @@
     </row>
     <row r="13" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="23">
         <v>0</v>
@@ -4175,7 +4166,7 @@
     </row>
     <row r="14" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="23">
         <v>0</v>
@@ -4223,7 +4214,7 @@
     </row>
     <row r="15" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="23">
         <v>4.2861136999068031E-2</v>
@@ -4271,7 +4262,7 @@
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="23">
         <v>0.1224070384497051</v>
@@ -4319,7 +4310,7 @@
     </row>
     <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="23">
         <v>0</v>
@@ -4367,7 +4358,7 @@
     </row>
     <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="23">
         <v>0</v>
@@ -4415,7 +4406,7 @@
     </row>
     <row r="19" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="23">
         <v>0</v>
@@ -4463,7 +4454,7 @@
     </row>
     <row r="20" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="23">
         <v>0.11072460391425908</v>
@@ -4511,7 +4502,7 @@
     </row>
     <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="23">
         <v>0</v>
@@ -4559,7 +4550,7 @@
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="23">
         <v>0</v>
@@ -4607,7 +4598,7 @@
     </row>
     <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="23">
         <v>0</v>
@@ -4655,7 +4646,7 @@
     </row>
     <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="26">
         <v>2.3598728952299282</v>
@@ -4703,7 +4694,7 @@
     </row>
     <row r="25" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="28">
         <v>94.99999998121919</v>
@@ -4752,7 +4743,7 @@
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -4760,7 +4751,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="I28" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="31"/>
       <c r="K28" s="31"/>
@@ -4770,48 +4761,48 @@
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="D29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="F29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="20" t="s">
+      <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="L29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="M29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="20" t="s">
+      <c r="N29" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N29" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A30" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="23">
         <v>0.13929869524697111</v>
@@ -4853,7 +4844,7 @@
     </row>
     <row r="31" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="23">
         <v>0.53626425908667286</v>
@@ -4901,7 +4892,7 @@
     </row>
     <row r="32" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="23">
         <v>3.990981717270381E-2</v>
@@ -4949,7 +4940,7 @@
     </row>
     <row r="33" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33" s="23">
         <v>0</v>
@@ -4997,7 +4988,7 @@
     </row>
     <row r="34" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="23">
         <v>0</v>
@@ -5045,7 +5036,7 @@
     </row>
     <row r="35" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="23">
         <v>2.9603901584342961E-2</v>
@@ -5093,7 +5084,7 @@
     </row>
     <row r="36" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="23">
         <v>4.3985752378274005E-2</v>
@@ -5141,7 +5132,7 @@
     </row>
     <row r="37" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="23">
         <v>0</v>
@@ -5189,7 +5180,7 @@
     </row>
     <row r="38" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="23">
         <v>0</v>
@@ -5237,7 +5228,7 @@
     </row>
     <row r="39" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="23">
         <v>4.2861136999068031E-2</v>
@@ -5285,7 +5276,7 @@
     </row>
     <row r="40" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="23">
         <v>5.7351833617708139E-2</v>
@@ -5332,7 +5323,7 @@
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="23">
         <v>0</v>
@@ -5379,7 +5370,7 @@
     </row>
     <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="23">
         <v>0</v>
@@ -5426,7 +5417,7 @@
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A43" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="23">
         <v>0</v>
@@ -5467,7 +5458,7 @@
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A44" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="23">
         <v>0.11072460391425908</v>
@@ -5508,7 +5499,7 @@
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A45" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="23">
         <v>0</v>
@@ -5549,7 +5540,7 @@
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A46" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="23">
         <v>0</v>
@@ -5590,7 +5581,7 @@
     </row>
     <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="23">
         <v>0</v>
@@ -5638,7 +5629,7 @@
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A48" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="26">
         <v>2.4663402732609487</v>
@@ -5679,7 +5670,7 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A49" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="28">
         <v>96.999999987266222</v>
@@ -6512,13 +6503,13 @@
     </row>
     <row r="3" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
       <c r="B4" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -6526,7 +6517,7 @@
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="I4" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
@@ -6536,48 +6527,48 @@
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I5" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="K5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="M5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="23">
         <v>0</v>
@@ -6625,7 +6616,7 @@
     </row>
     <row r="7" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="23">
         <v>0.45784622382024798</v>
@@ -6673,7 +6664,7 @@
     </row>
     <row r="8" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="23">
         <v>0.17986725663716813</v>
@@ -6721,7 +6712,7 @@
     </row>
     <row r="9" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="23">
         <v>5.514217165264885E-5</v>
@@ -6769,7 +6760,7 @@
     </row>
     <row r="10" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="23">
         <v>0</v>
@@ -6817,7 +6808,7 @@
     </row>
     <row r="11" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="23">
         <v>4.3052733689287345E-2</v>
@@ -6865,7 +6856,7 @@
     </row>
     <row r="12" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="23">
         <v>0</v>
@@ -6913,7 +6904,7 @@
     </row>
     <row r="13" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="23">
         <v>0</v>
@@ -6961,7 +6952,7 @@
     </row>
     <row r="14" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="23">
         <v>3.3359800800949475E-2</v>
@@ -7009,7 +7000,7 @@
     </row>
     <row r="15" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="23">
         <v>3.4141811427947116E-2</v>
@@ -7057,7 +7048,7 @@
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="23">
         <v>0.16940892010066935</v>
@@ -7105,7 +7096,7 @@
     </row>
     <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="23">
         <v>0</v>
@@ -7153,7 +7144,7 @@
     </row>
     <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="23">
         <v>0</v>
@@ -7201,7 +7192,7 @@
     </row>
     <row r="19" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="23">
         <v>0</v>
@@ -7249,7 +7240,7 @@
     </row>
     <row r="20" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="23">
         <v>6.2820933027422698E-2</v>
@@ -7297,7 +7288,7 @@
     </row>
     <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="23">
         <v>0</v>
@@ -7345,7 +7336,7 @@
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="23">
         <v>1.9447175789348032E-2</v>
@@ -7393,7 +7384,7 @@
     </row>
     <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="23">
         <v>0</v>
@@ -7441,7 +7432,7 @@
     </row>
     <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="26">
         <v>2.2571142372530715</v>
@@ -7489,7 +7480,7 @@
     </row>
     <row r="25" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="28">
         <v>91.015161291112832</v>
@@ -7538,7 +7529,7 @@
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -7546,7 +7537,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="I28" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="31"/>
       <c r="K28" s="31"/>
@@ -7556,48 +7547,48 @@
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="D29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="F29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="20" t="s">
+      <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="L29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="M29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="20" t="s">
+      <c r="N29" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N29" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A30" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="23">
         <v>0</v>
@@ -7639,7 +7630,7 @@
     </row>
     <row r="31" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="23">
         <v>0.21544848356650281</v>
@@ -7687,7 +7678,7 @@
     </row>
     <row r="32" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="23">
         <v>0.2163647475612252</v>
@@ -7735,7 +7726,7 @@
     </row>
     <row r="33" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33" s="23">
         <v>0</v>
@@ -7783,7 +7774,7 @@
     </row>
     <row r="34" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="23">
         <v>0</v>
@@ -7831,7 +7822,7 @@
     </row>
     <row r="35" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="23">
         <v>0</v>
@@ -7879,7 +7870,7 @@
     </row>
     <row r="36" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="23">
         <v>0</v>
@@ -7927,7 +7918,7 @@
     </row>
     <row r="37" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="23">
         <v>0</v>
@@ -7975,7 +7966,7 @@
     </row>
     <row r="38" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="23">
         <v>0</v>
@@ -8023,7 +8014,7 @@
     </row>
     <row r="39" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="23">
         <v>0</v>
@@ -8071,7 +8062,7 @@
     </row>
     <row r="40" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="23">
         <v>7.833986219933213E-2</v>
@@ -8118,7 +8109,7 @@
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="23">
         <v>0</v>
@@ -8165,7 +8156,7 @@
     </row>
     <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="23">
         <v>0</v>
@@ -8212,7 +8203,7 @@
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A43" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="23">
         <v>0</v>
@@ -8253,7 +8244,7 @@
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A44" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="23">
         <v>0.31482232552868922</v>
@@ -8294,7 +8285,7 @@
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A45" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="23">
         <v>0</v>
@@ -8335,7 +8326,7 @@
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A46" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="23">
         <v>0.17502458210422814</v>
@@ -8376,7 +8367,7 @@
     </row>
     <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="23">
         <v>0</v>
@@ -8424,7 +8415,7 @@
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A48" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="26">
         <v>2.2404053836860762</v>
@@ -8465,7 +8456,7 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A49" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="28">
         <v>94.000000299863331</v>
@@ -9297,13 +9288,13 @@
     </row>
     <row r="3" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
       <c r="B4" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -9311,7 +9302,7 @@
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="I4" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
@@ -9321,48 +9312,48 @@
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I5" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="K5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="M5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="23">
         <v>0.11346140339141937</v>
@@ -9410,7 +9401,7 @@
     </row>
     <row r="7" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="23">
         <v>0.1761179676306982</v>
@@ -9458,7 +9449,7 @@
     </row>
     <row r="8" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="23">
         <v>0.13053325758445614</v>
@@ -9506,7 +9497,7 @@
     </row>
     <row r="9" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="23">
         <v>8.9352802405765541E-2</v>
@@ -9554,7 +9545,7 @@
     </row>
     <row r="10" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="23">
         <v>0</v>
@@ -9602,7 +9593,7 @@
     </row>
     <row r="11" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="23">
         <v>1.7873070116803381E-2</v>
@@ -9650,7 +9641,7 @@
     </row>
     <row r="12" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="23">
         <v>0</v>
@@ -9698,7 +9689,7 @@
     </row>
     <row r="13" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="23">
         <v>0</v>
@@ -9746,7 +9737,7 @@
     </row>
     <row r="14" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="23">
         <v>2.2721354435037044E-2</v>
@@ -9794,7 +9785,7 @@
     </row>
     <row r="15" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="23">
         <v>8.4447176912069571E-2</v>
@@ -9842,7 +9833,7 @@
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="23">
         <v>4.169892802947324E-2</v>
@@ -9890,7 +9881,7 @@
     </row>
     <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="23">
         <v>7.96934580916841E-2</v>
@@ -9938,7 +9929,7 @@
     </row>
     <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="23">
         <v>0</v>
@@ -9986,7 +9977,7 @@
     </row>
     <row r="19" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="23">
         <v>0</v>
@@ -10034,7 +10025,7 @@
     </row>
     <row r="20" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="23">
         <v>0.1682515636214145</v>
@@ -10082,7 +10073,7 @@
     </row>
     <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="23">
         <v>6.5720938608164858E-2</v>
@@ -10130,7 +10121,7 @@
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="23">
         <v>1.0128079173014021E-2</v>
@@ -10178,7 +10169,7 @@
     </row>
     <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="23">
         <v>0</v>
@@ -10226,7 +10217,7 @@
     </row>
     <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="26">
         <v>2.3879284427767251</v>
@@ -10274,7 +10265,7 @@
     </row>
     <row r="25" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="28">
         <v>95</v>
@@ -10323,7 +10314,7 @@
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -10331,7 +10322,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="I28" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="31"/>
       <c r="K28" s="31"/>
@@ -10341,48 +10332,48 @@
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="D29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="F29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="20" t="s">
+      <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="L29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="M29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="20" t="s">
+      <c r="N29" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N29" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A30" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="23">
         <v>0.10819840760298839</v>
@@ -10424,7 +10415,7 @@
     </row>
     <row r="31" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="23">
         <v>0.25339819391721502</v>
@@ -10472,7 +10463,7 @@
     </row>
     <row r="32" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="23">
         <v>0.12546755444331839</v>
@@ -10520,7 +10511,7 @@
     </row>
     <row r="33" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33" s="23">
         <v>8.5599928806146988E-2</v>
@@ -10568,7 +10559,7 @@
     </row>
     <row r="34" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="23">
         <v>0</v>
@@ -10616,7 +10607,7 @@
     </row>
     <row r="35" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="23">
         <v>2.5913057934956445E-2</v>
@@ -10664,7 +10655,7 @@
     </row>
     <row r="36" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="23">
         <v>0</v>
@@ -10712,7 +10703,7 @@
     </row>
     <row r="37" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="23">
         <v>0</v>
@@ -10760,7 +10751,7 @@
     </row>
     <row r="38" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="23">
         <v>8.813231025538203E-3</v>
@@ -10808,7 +10799,7 @@
     </row>
     <row r="39" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="23">
         <v>7.9927785589466976E-2</v>
@@ -10856,7 +10847,7 @@
     </row>
     <row r="40" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="23">
         <v>0</v>
@@ -10903,7 +10894,7 @@
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="23">
         <v>6.5068518146008072E-2</v>
@@ -10950,7 +10941,7 @@
     </row>
     <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="23">
         <v>0</v>
@@ -10997,7 +10988,7 @@
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A43" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="23">
         <v>0</v>
@@ -11038,7 +11029,7 @@
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A44" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="23">
         <v>0.17462199089806596</v>
@@ -11079,7 +11070,7 @@
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A45" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="23">
         <v>6.8152241495472277E-2</v>
@@ -11120,7 +11111,7 @@
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A46" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="23">
         <v>4.8390901408232861E-3</v>
@@ -11161,7 +11152,7 @@
     </row>
     <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="23">
         <v>0</v>
@@ -11209,7 +11200,7 @@
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A48" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="26">
         <v>2.44490181918396</v>
@@ -11250,7 +11241,7 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A49" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="28">
         <v>97.999999999999986</v>
@@ -12082,13 +12073,13 @@
     </row>
     <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
       <c r="B4" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -12096,7 +12087,7 @@
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="I4" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
@@ -12106,48 +12097,48 @@
     </row>
     <row r="5" spans="1:14" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I5" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="K5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="M5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A6" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="23">
         <v>0.24581500078473237</v>
@@ -12189,7 +12180,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A7" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="23">
         <v>0.36634062332347123</v>
@@ -12231,7 +12222,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A8" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="23">
         <v>3.30736878814775E-2</v>
@@ -12273,7 +12264,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A9" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="23">
         <v>0</v>
@@ -12315,7 +12306,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="23">
         <v>0</v>
@@ -12357,7 +12348,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A11" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="23">
         <v>2.6545030806351917E-2</v>
@@ -12399,7 +12390,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A12" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="23">
         <v>0.11980028520786347</v>
@@ -12441,7 +12432,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A13" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="23">
         <v>0</v>
@@ -12483,7 +12474,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A14" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="23">
         <v>0</v>
@@ -12525,7 +12516,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A15" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="23">
         <v>0</v>
@@ -12567,7 +12558,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A16" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="23">
         <v>0.10518607419719359</v>
@@ -12608,7 +12599,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="23">
         <v>0</v>
@@ -12649,7 +12640,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A18" s="25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="23">
         <v>0</v>
@@ -12690,7 +12681,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="23">
         <v>0</v>
@@ -12731,7 +12722,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A20" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="23">
         <v>0</v>
@@ -12772,7 +12763,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A21" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="23">
         <v>0.10323929779890985</v>
@@ -12813,7 +12804,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A22" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="23">
         <v>0</v>
@@ -12854,7 +12845,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A23" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="23">
         <v>0</v>
@@ -12895,7 +12886,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A24" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="26">
         <v>2.2559673073236768</v>
@@ -12936,7 +12927,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="28">
         <v>91.000000025803217</v>
@@ -12978,7 +12969,7 @@
     <row r="28" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -12986,7 +12977,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="I28" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="31"/>
       <c r="K28" s="31"/>
@@ -12996,48 +12987,48 @@
     </row>
     <row r="29" spans="1:14" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="D29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="F29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="20" t="s">
+      <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="L29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="M29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="20" t="s">
+      <c r="N29" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N29" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A30" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="23">
         <v>0.24581500078473237</v>
@@ -13078,7 +13069,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A31" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="23">
         <v>0.3663416233234712</v>
@@ -13119,7 +13110,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A32" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="23">
         <v>0.13533751869954713</v>
@@ -13160,7 +13151,7 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A33" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33" s="23">
         <v>0</v>
@@ -13201,7 +13192,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A34" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="23">
         <v>0</v>
@@ -13242,7 +13233,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A35" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="23">
         <v>2.6545030806351917E-2</v>
@@ -13283,7 +13274,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A36" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="23">
         <v>5.6182483267950299E-2</v>
@@ -13324,7 +13315,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="23">
         <v>0</v>
@@ -13365,7 +13356,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A38" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="23">
         <v>6.3000952375921668E-2</v>
@@ -13406,7 +13397,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A39" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="23">
         <v>0</v>
@@ -13447,7 +13438,7 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A40" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="23">
         <v>0</v>
@@ -13488,7 +13479,7 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A41" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="23">
         <v>0</v>
@@ -13529,7 +13520,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A42" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="23">
         <v>0</v>
@@ -13570,7 +13561,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A43" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="23">
         <v>0</v>
@@ -13611,7 +13602,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A44" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="23">
         <v>0</v>
@@ -13652,7 +13643,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A45" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="23">
         <v>0.10677839074202548</v>
@@ -13693,7 +13684,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A46" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="23">
         <v>0</v>
@@ -13734,7 +13725,7 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A47" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="23">
         <v>0</v>
@@ -13775,7 +13766,7 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A48" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="26">
         <v>2.5048829491088593</v>
@@ -13816,7 +13807,7 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A49" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="28">
         <v>95.000107999999997</v>
@@ -13896,13 +13887,13 @@
     </row>
     <row r="3" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
       <c r="B4" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="31"/>
@@ -13910,7 +13901,7 @@
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="I4" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
@@ -13920,48 +13911,48 @@
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I5" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="K5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="M5" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="23">
         <v>5.9691196028287659E-2</v>
@@ -14009,7 +14000,7 @@
     </row>
     <row r="7" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="23">
         <v>0.65013907489990008</v>
@@ -14057,7 +14048,7 @@
     </row>
     <row r="8" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="23">
         <v>0</v>
@@ -14105,7 +14096,7 @@
     </row>
     <row r="9" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="23">
         <v>0</v>
@@ -14153,7 +14144,7 @@
     </row>
     <row r="10" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="23">
         <v>0</v>
@@ -14201,7 +14192,7 @@
     </row>
     <row r="11" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="23">
         <v>8.3826147820382488E-2</v>
@@ -14249,7 +14240,7 @@
     </row>
     <row r="12" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="23">
         <v>0</v>
@@ -14297,7 +14288,7 @@
     </row>
     <row r="13" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="23">
         <v>0</v>
@@ -14345,7 +14336,7 @@
     </row>
     <row r="14" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="23">
         <v>4.2243471158183952E-12</v>
@@ -14393,7 +14384,7 @@
     </row>
     <row r="15" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="23">
         <v>0</v>
@@ -14441,7 +14432,7 @@
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="23">
         <v>0.20634357820228202</v>
@@ -14489,7 +14480,7 @@
     </row>
     <row r="17" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="23">
         <v>8.2701217280467648E-14</v>
@@ -14537,7 +14528,7 @@
     </row>
     <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="23">
         <v>0</v>
@@ -14585,7 +14576,7 @@
     </row>
     <row r="19" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="23">
         <v>0</v>
@@ -14633,7 +14624,7 @@
     </row>
     <row r="20" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="23">
         <v>0</v>
@@ -14681,7 +14672,7 @@
     </row>
     <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="23">
         <v>0</v>
@@ -14729,7 +14720,7 @@
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" s="23">
         <v>1.177178771520086E-12</v>
@@ -14777,7 +14768,7 @@
     </row>
     <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23" s="23">
         <v>0</v>
@@ -14825,7 +14816,7 @@
     </row>
     <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24" s="26">
         <v>2.2802389000653194</v>
@@ -14873,7 +14864,7 @@
     </row>
     <row r="25" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="28">
         <v>92.000000236352349</v>
@@ -14922,7 +14913,7 @@
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
       <c r="B28" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -14930,7 +14921,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="31"/>
       <c r="I28" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="31"/>
       <c r="K28" s="31"/>
@@ -14940,48 +14931,48 @@
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="D29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="F29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="20" t="s">
+      <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="20" t="s">
+      <c r="L29" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L29" s="20" t="s">
+      <c r="M29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="20" t="s">
+      <c r="N29" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N29" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A30" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="23">
         <v>0.27480834537642607</v>
@@ -15023,7 +15014,7 @@
     </row>
     <row r="31" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="23">
         <v>0.5539409117748253</v>
@@ -15071,7 +15062,7 @@
     </row>
     <row r="32" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="23">
         <v>0</v>
@@ -15119,7 +15110,7 @@
     </row>
     <row r="33" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B33" s="23">
         <v>0</v>
@@ -15167,7 +15158,7 @@
     </row>
     <row r="34" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="23">
         <v>0</v>
@@ -15215,7 +15206,7 @@
     </row>
     <row r="35" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="23">
         <v>8.2024809478008359E-2</v>
@@ -15263,7 +15254,7 @@
     </row>
     <row r="36" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="23">
         <v>0</v>
@@ -15311,7 +15302,7 @@
     </row>
     <row r="37" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="23">
         <v>0</v>
@@ -15359,7 +15350,7 @@
     </row>
     <row r="38" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="23">
         <v>0</v>
@@ -15407,7 +15398,7 @@
     </row>
     <row r="39" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="23">
         <v>0</v>
@@ -15455,7 +15446,7 @@
     </row>
     <row r="40" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="23">
         <v>8.9225933370740265E-2</v>
@@ -15502,7 +15493,7 @@
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="23">
         <v>0</v>
@@ -15549,7 +15540,7 @@
     </row>
     <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="23">
         <v>0</v>
@@ -15596,7 +15587,7 @@
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A43" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="23">
         <v>0</v>
@@ -15637,7 +15628,7 @@
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A44" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="23">
         <v>0</v>
@@ -15678,7 +15669,7 @@
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A45" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="23">
         <v>0</v>
@@ -15719,7 +15710,7 @@
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A46" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="23">
         <v>0</v>
@@ -15760,7 +15751,7 @@
     </row>
     <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="23">
         <v>0</v>
@@ -15808,7 +15799,7 @@
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A48" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="26">
         <v>2.4364032993835236</v>
@@ -15849,7 +15840,7 @@
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A49" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="28">
         <v>95</v>
@@ -15923,7 +15914,7 @@
     <row r="52" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="12"/>
       <c r="B52" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C52" s="31"/>
       <c r="D52" s="31"/>
@@ -15931,7 +15922,7 @@
       <c r="F52" s="31"/>
       <c r="G52" s="31"/>
       <c r="I52" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J52" s="31"/>
       <c r="K52" s="31"/>
@@ -15941,48 +15932,48 @@
     </row>
     <row r="53" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A53" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B53" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C53" s="20" t="s">
+      <c r="D53" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D53" s="20" t="s">
+      <c r="E53" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E53" s="20" t="s">
+      <c r="F53" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F53" s="20" t="s">
+      <c r="G53" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G53" s="21" t="s">
-        <v>19</v>
-      </c>
       <c r="I53" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="J53" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J53" s="20" t="s">
+      <c r="K53" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K53" s="20" t="s">
+      <c r="L53" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L53" s="20" t="s">
+      <c r="M53" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="M53" s="20" t="s">
+      <c r="N53" s="21" t="s">
         <v>18</v>
-      </c>
-      <c r="N53" s="21" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="54" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B54" s="23">
         <v>0.41821978960375611</v>
@@ -16031,7 +16022,7 @@
     </row>
     <row r="55" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A55" s="22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B55" s="23">
         <v>0.48980879845072295</v>
@@ -16080,7 +16071,7 @@
     </row>
     <row r="56" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B56" s="23">
         <v>0</v>
@@ -16129,7 +16120,7 @@
     </row>
     <row r="57" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A57" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B57" s="23">
         <v>0</v>
@@ -16178,7 +16169,7 @@
     </row>
     <row r="58" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A58" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B58" s="23">
         <v>0</v>
@@ -16227,7 +16218,7 @@
     </row>
     <row r="59" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A59" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B59" s="23">
         <v>8.0823920250636769E-2</v>
@@ -16276,7 +16267,7 @@
     </row>
     <row r="60" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A60" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B60" s="23">
         <v>0</v>
@@ -16325,7 +16316,7 @@
     </row>
     <row r="61" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A61" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B61" s="23">
         <v>0</v>
@@ -16374,7 +16365,7 @@
     </row>
     <row r="62" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A62" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B62" s="23">
         <v>0</v>
@@ -16423,7 +16414,7 @@
     </row>
     <row r="63" spans="1:23" s="9" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A63" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B63" s="23">
         <v>0</v>
@@ -16472,7 +16463,7 @@
     </row>
     <row r="64" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A64" s="25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B64" s="23">
         <v>1.1147491694884144E-2</v>
@@ -16520,7 +16511,7 @@
     </row>
     <row r="65" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B65" s="23">
         <v>0</v>
@@ -16568,7 +16559,7 @@
     </row>
     <row r="66" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A66" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B66" s="23">
         <v>0</v>
@@ -16616,7 +16607,7 @@
     </row>
     <row r="67" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A67" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B67" s="23">
         <v>0</v>
@@ -16664,7 +16655,7 @@
     </row>
     <row r="68" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A68" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B68" s="23">
         <v>0</v>
@@ -16712,7 +16703,7 @@
     </row>
     <row r="69" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A69" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B69" s="23">
         <v>0</v>
@@ -16760,7 +16751,7 @@
     </row>
     <row r="70" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A70" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B70" s="23">
         <v>0</v>
@@ -16808,7 +16799,7 @@
     </row>
     <row r="71" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A71" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B71" s="23">
         <v>0</v>
@@ -16856,7 +16847,7 @@
     </row>
     <row r="72" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A72" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B72" s="26">
         <v>2.5405129081006703</v>
@@ -16904,7 +16895,7 @@
     </row>
     <row r="73" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A73" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B73" s="28">
         <v>97</v>

</xml_diff>

<commit_message>
Se suben las imágenes de carga de Agosto
</commit_message>
<xml_diff>
--- a/storage/app/pdfs/blending_asia_components.xlsx
+++ b/storage/app/pdfs/blending_asia_components.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://faro90mx-my.sharepoint.com/personal/rfavela_hcx_mx/Documents/F90/Operacion/Proyectos/Proyectos en curso/US Grains 013 (Analisis Global)/Asia Africa/1. Informacion AsiaAfrica/2. Blending/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodrigofavela/Desktop/Update Blending EIH/BLENDING/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{C8AD3F2B-3DD6-0C4F-A3F6-C4486412BC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B48AAAD5-5CA5-4540-BAA1-E8C4D309E7EA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D77601-9C28-3F42-82F3-A565A6C4E308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4900" yWindow="4340" windowWidth="23280" windowHeight="12480" tabRatio="853" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
+    <workbookView xWindow="6920" yWindow="4200" windowWidth="23400" windowHeight="17400" tabRatio="853" activeTab="5" xr2:uid="{AD60D5F5-4EC3-4F16-A51A-8F435208B142}"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="7" r:id="rId1"/>
@@ -457,11 +457,11 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="4" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -885,12 +885,12 @@
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="31" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="30"/>
+      <c r="A6" s="31"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
@@ -1048,22 +1048,22 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="I4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
@@ -1941,40 +1941,40 @@
         <v>37</v>
       </c>
       <c r="B24" s="26">
-        <v>2.2233780546404009</v>
+        <v>2.0102800515825239</v>
       </c>
       <c r="C24" s="26">
-        <v>2.22337807404501</v>
+        <v>2.0102800709871329</v>
       </c>
       <c r="D24" s="26">
-        <v>2.2233187541917427</v>
+        <v>2.0102207511338657</v>
       </c>
       <c r="E24" s="26">
-        <v>2.2233732214964999</v>
+        <v>2.0102752184386228</v>
       </c>
       <c r="F24" s="26">
-        <v>2.2233780435079602</v>
+        <v>2.0102800404500831</v>
       </c>
       <c r="G24" s="26">
-        <v>2.2232910218824578</v>
+        <v>2.0101930188245807</v>
       </c>
       <c r="I24" s="27">
-        <v>2.2233780546404009</v>
+        <v>2.0102800515825239</v>
       </c>
       <c r="J24" s="27">
-        <v>1.9686677937337684</v>
+        <v>1.7555697906758914</v>
       </c>
       <c r="K24" s="27">
-        <v>1.8257584046450617</v>
+        <v>1.6126604015871846</v>
       </c>
       <c r="L24" s="27">
-        <v>1.6777991483585706</v>
+        <v>1.4647011453006935</v>
       </c>
       <c r="M24" s="27">
-        <v>1.6114710132471082</v>
+        <v>1.3983730101892311</v>
       </c>
       <c r="N24" s="27">
-        <v>1.5300386368571033</v>
+        <v>1.3169406337992262</v>
       </c>
       <c r="Q24" s="13"/>
       <c r="R24" s="13"/>
@@ -2027,22 +2027,22 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="I28" s="31" t="s">
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="I28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
     </row>
     <row r="29" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
@@ -2957,40 +2957,40 @@
         <v>37</v>
       </c>
       <c r="B48" s="26">
-        <v>2.4212259613369422</v>
+        <v>2.2081279582790652</v>
       </c>
       <c r="C48" s="26">
-        <v>2.4212259378201062</v>
+        <v>2.2081279347622291</v>
       </c>
       <c r="D48" s="26">
-        <v>2.4212259514762211</v>
+        <v>2.208127948418344</v>
       </c>
       <c r="E48" s="26">
-        <v>2.4212259377038192</v>
+        <v>2.2081279346459421</v>
       </c>
       <c r="F48" s="26">
-        <v>2.421225933729525</v>
+        <v>2.2081279306716479</v>
       </c>
       <c r="G48" s="26">
-        <v>2.4212259453718046</v>
+        <v>2.2081279423139275</v>
       </c>
       <c r="I48" s="27">
-        <v>2.4212259613369422</v>
+        <v>2.2081279582790652</v>
       </c>
       <c r="J48" s="27">
-        <v>2.3442791995026275</v>
+        <v>2.1311811964447505</v>
       </c>
       <c r="K48" s="27">
-        <v>2.2648820958749467</v>
+        <v>2.0517840928170696</v>
       </c>
       <c r="L48" s="27">
-        <v>2.1798484890675409</v>
+        <v>1.9667504860096638</v>
       </c>
       <c r="M48" s="27">
-        <v>2.0902002854769952</v>
+        <v>1.8771022824191181</v>
       </c>
       <c r="N48" s="27">
-        <v>1.9840605379170211</v>
+        <v>1.770962534859144</v>
       </c>
       <c r="Q48" s="13"/>
       <c r="R48" s="13"/>
@@ -3722,22 +3722,22 @@
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="I4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
@@ -4649,40 +4649,40 @@
         <v>37</v>
       </c>
       <c r="B24" s="26">
-        <v>2.3598728952299282</v>
+        <v>2.1467748921720511</v>
       </c>
       <c r="C24" s="26">
-        <v>2.3598728925217616</v>
+        <v>2.1467748894638845</v>
       </c>
       <c r="D24" s="26">
-        <v>2.3598728922277417</v>
+        <v>2.1467748891698646</v>
       </c>
       <c r="E24" s="26">
-        <v>2.3598728927562349</v>
+        <v>2.1467748896983578</v>
       </c>
       <c r="F24" s="26">
-        <v>2.3598728943973621</v>
+        <v>2.1467748913394851</v>
       </c>
       <c r="G24" s="26">
-        <v>2.3598728945610059</v>
+        <v>2.1467748915031288</v>
       </c>
       <c r="I24" s="27">
-        <v>2.3598728952299282</v>
+        <v>2.1467748921720511</v>
       </c>
       <c r="J24" s="27">
-        <v>2.2318883411423487</v>
+        <v>2.0187903380844716</v>
       </c>
       <c r="K24" s="27">
-        <v>2.163589890801541</v>
+        <v>1.9504918877436639</v>
       </c>
       <c r="L24" s="27">
-        <v>2.1016246801356506</v>
+        <v>1.8885266770777736</v>
       </c>
       <c r="M24" s="27">
-        <v>2.0248512939943479</v>
+        <v>1.8117532909364709</v>
       </c>
       <c r="N24" s="27">
-        <v>1.9749100326913309</v>
+        <v>1.7618120296334538</v>
       </c>
       <c r="Q24" s="17"/>
       <c r="R24" s="14"/>
@@ -4742,22 +4742,22 @@
     </row>
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="I28" s="31" t="s">
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="I28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
@@ -5632,40 +5632,40 @@
         <v>37</v>
       </c>
       <c r="B48" s="26">
-        <v>2.4663402732609487</v>
+        <v>2.2532422702030717</v>
       </c>
       <c r="C48" s="26">
-        <v>2.466340272310144</v>
+        <v>2.2532422692522669</v>
       </c>
       <c r="D48" s="26">
-        <v>2.4663402742272051</v>
+        <v>2.2532422711693281</v>
       </c>
       <c r="E48" s="26">
-        <v>2.4663402723101435</v>
+        <v>2.2532422692522664</v>
       </c>
       <c r="F48" s="26">
-        <v>2.4663402737821598</v>
+        <v>2.2532422707242827</v>
       </c>
       <c r="G48" s="26">
-        <v>2.4663402742297373</v>
+        <v>2.2532422711718603</v>
       </c>
       <c r="I48" s="27">
-        <v>2.4663402732609487</v>
+        <v>2.2532422702030717</v>
       </c>
       <c r="J48" s="27">
-        <v>2.345457188550792</v>
+        <v>2.1323591854929149</v>
       </c>
       <c r="K48" s="27">
-        <v>2.2491838239658577</v>
+        <v>2.0360858209079806</v>
       </c>
       <c r="L48" s="27">
-        <v>2.1865982936872435</v>
+        <v>1.9735002906293664</v>
       </c>
       <c r="M48" s="27">
-        <v>2.1156867000699586</v>
+        <v>1.9025886970120816</v>
       </c>
       <c r="N48" s="27">
-        <v>2.032820865866801</v>
+        <v>1.8197228628089239</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
@@ -6508,22 +6508,22 @@
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="I4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
@@ -7334,7 +7334,7 @@
       <c r="V21" s="13"/>
       <c r="W21" s="13"/>
     </row>
-    <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A22" s="25" t="s">
         <v>35</v>
       </c>
@@ -7374,15 +7374,8 @@
       <c r="N22" s="24">
         <v>0.12580491642084499</v>
       </c>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
-      <c r="T22" s="13"/>
-      <c r="U22" s="13"/>
-      <c r="V22" s="13"/>
-      <c r="W22" s="13"/>
-    </row>
-    <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A23" s="25" t="s">
         <v>36</v>
       </c>
@@ -7422,63 +7415,49 @@
       <c r="N23" s="24">
         <v>0.3</v>
       </c>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
-      <c r="V23" s="13"/>
-      <c r="W23" s="13"/>
-    </row>
-    <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A24" s="25" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="26">
-        <v>2.2571142372530715</v>
+        <v>2.0273073806281992</v>
       </c>
       <c r="C24" s="26">
-        <v>2.2570254479822482</v>
+        <v>2.027267156422242</v>
       </c>
       <c r="D24" s="26">
-        <v>2.2570131002441682</v>
+        <v>2.0273073009589346</v>
       </c>
       <c r="E24" s="26">
-        <v>2.257112094115111</v>
+        <v>2.027307414372618</v>
       </c>
       <c r="F24" s="26">
-        <v>2.2571085830844777</v>
+        <v>2.0273072255755631</v>
       </c>
       <c r="G24" s="26">
-        <v>2.2571175255962008</v>
+        <v>2.02730737945617</v>
       </c>
       <c r="I24" s="27">
-        <v>2.2571142372530715</v>
+        <v>2.0273073806281992</v>
       </c>
       <c r="J24" s="27">
-        <v>2.1368280904684385</v>
+        <v>1.9719427731834966</v>
       </c>
       <c r="K24" s="27">
-        <v>2.0943373177789484</v>
+        <v>1.9266100818575529</v>
       </c>
       <c r="L24" s="27">
-        <v>2.0500875023791498</v>
+        <v>1.8728352871862399</v>
       </c>
       <c r="M24" s="27">
-        <v>2.0012385964408801</v>
+        <v>1.8466229881305933</v>
       </c>
       <c r="N24" s="27">
-        <v>1.9494347893778274</v>
-      </c>
-      <c r="Q24" s="17"/>
-      <c r="R24" s="14"/>
-      <c r="S24" s="14"/>
-      <c r="T24" s="14"/>
-      <c r="U24" s="14"/>
-      <c r="V24" s="14"/>
-      <c r="W24" s="14"/>
-    </row>
-    <row r="25" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+        <v>1.8667033050074195</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A25" s="25" t="s">
         <v>38</v>
       </c>
@@ -7518,32 +7497,25 @@
       <c r="N25" s="29">
         <v>95.315902875997097</v>
       </c>
-      <c r="Q25" s="16"/>
-      <c r="R25" s="15"/>
-      <c r="S25" s="15"/>
-      <c r="T25" s="15"/>
-      <c r="U25" s="15"/>
-      <c r="V25" s="15"/>
-      <c r="W25" s="15"/>
     </row>
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="I28" s="31" t="s">
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="I28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
@@ -8418,40 +8390,40 @@
         <v>37</v>
       </c>
       <c r="B48" s="26">
-        <v>2.2404053836860762</v>
+        <v>2.0440162341951944</v>
       </c>
       <c r="C48" s="26">
-        <v>2.2403651594801191</v>
+        <v>2.0439274449243712</v>
       </c>
       <c r="D48" s="26">
-        <v>2.2404053040168117</v>
+        <v>2.0439150971862912</v>
       </c>
       <c r="E48" s="26">
-        <v>2.240405417430495</v>
+        <v>2.044014091057234</v>
       </c>
       <c r="F48" s="26">
-        <v>2.2404052286334402</v>
+        <v>2.0440105800266006</v>
       </c>
       <c r="G48" s="26">
-        <v>2.2404053825140471</v>
+        <v>2.0440195225383238</v>
       </c>
       <c r="I48" s="27">
-        <v>2.2404053836860762</v>
+        <v>2.0440162341951944</v>
       </c>
       <c r="J48" s="27">
-        <v>2.1850407762413737</v>
+        <v>1.9237300874105614</v>
       </c>
       <c r="K48" s="27">
-        <v>2.13970808491543</v>
+        <v>1.8812393147210713</v>
       </c>
       <c r="L48" s="27">
-        <v>2.085933290244117</v>
+        <v>1.8369894993212728</v>
       </c>
       <c r="M48" s="27">
-        <v>2.0597209911884704</v>
+        <v>1.788140593383003</v>
       </c>
       <c r="N48" s="27">
-        <v>2.0798013080652966</v>
+        <v>1.7363367863199504</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
@@ -9293,22 +9265,22 @@
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="I4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
@@ -10220,40 +10192,40 @@
         <v>37</v>
       </c>
       <c r="B24" s="26">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="C24" s="26">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="D24" s="26">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="E24" s="26">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="F24" s="26">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="G24" s="26">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="I24" s="27">
-        <v>2.3879284427767251</v>
+        <v>2.174830439718848</v>
       </c>
       <c r="J24" s="27">
-        <v>2.3068763615741918</v>
+        <v>2.0937783585163148</v>
       </c>
       <c r="K24" s="27">
-        <v>2.2226398339398155</v>
+        <v>2.0095418308819384</v>
       </c>
       <c r="L24" s="27">
-        <v>2.1489030491685752</v>
+        <v>1.9358050461106981</v>
       </c>
       <c r="M24" s="27">
-        <v>2.0612976483579644</v>
+        <v>1.8481996453000873</v>
       </c>
       <c r="N24" s="27">
-        <v>1.9946873727919308</v>
+        <v>1.7815893697340537</v>
       </c>
       <c r="Q24" s="17"/>
       <c r="R24" s="14"/>
@@ -10313,22 +10285,22 @@
     </row>
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="I28" s="31" t="s">
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="I28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
@@ -11203,40 +11175,40 @@
         <v>37</v>
       </c>
       <c r="B48" s="26">
-        <v>2.44490181918396</v>
+        <v>2.2318038161260829</v>
       </c>
       <c r="C48" s="26">
-        <v>2.44490181918396</v>
+        <v>2.2318038161260829</v>
       </c>
       <c r="D48" s="26">
-        <v>2.444901866843129</v>
+        <v>2.231803863785252</v>
       </c>
       <c r="E48" s="26">
-        <v>2.4449018529225528</v>
+        <v>2.2318038498646757</v>
       </c>
       <c r="F48" s="26">
-        <v>2.444901776696176</v>
+        <v>2.231803773638299</v>
       </c>
       <c r="G48" s="26">
-        <v>2.4449017919051808</v>
+        <v>2.2318037888473037</v>
       </c>
       <c r="I48" s="27">
-        <v>2.4449018211633438</v>
+        <v>2.2318038181054667</v>
       </c>
       <c r="J48" s="27">
-        <v>2.4182181600637329</v>
+        <v>2.2051201570058558</v>
       </c>
       <c r="K48" s="27">
-        <v>2.3462413900693915</v>
+        <v>2.1331433870115144</v>
       </c>
       <c r="L48" s="27">
-        <v>2.3050940723700211</v>
+        <v>2.091996069312144</v>
       </c>
       <c r="M48" s="27">
-        <v>2.2101565605205264</v>
+        <v>1.9970585574626494</v>
       </c>
       <c r="N48" s="27">
-        <v>2.1168156893288601</v>
+        <v>1.903717686270983</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
@@ -12051,7 +12023,7 @@
   <sheetPr>
     <tabColor rgb="FFD18316"/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="26" style="8" bestFit="1" customWidth="1"/>
@@ -12078,22 +12050,22 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="I4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:14" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
@@ -12889,40 +12861,40 @@
         <v>37</v>
       </c>
       <c r="B24" s="26">
-        <v>2.2559673073236768</v>
+        <v>2.0428693042657997</v>
       </c>
       <c r="C24" s="26">
-        <v>2.255967310159257</v>
+        <v>2.0428693071013799</v>
       </c>
       <c r="D24" s="26">
-        <v>2.2559673061213381</v>
+        <v>2.042869303063461</v>
       </c>
       <c r="E24" s="26">
-        <v>2.2559673076762339</v>
+        <v>2.0428693046183568</v>
       </c>
       <c r="F24" s="26">
-        <v>2.2559673137432084</v>
+        <v>2.0428693106853313</v>
       </c>
       <c r="G24" s="26">
-        <v>2.2559673048962465</v>
+        <v>2.0428693018383695</v>
       </c>
       <c r="I24" s="27">
-        <v>2.2559673073236768</v>
+        <v>2.0428693042657997</v>
       </c>
       <c r="J24" s="27">
-        <v>2.1227234174730998</v>
+        <v>1.9096254144152227</v>
       </c>
       <c r="K24" s="27">
-        <v>2.0067185959814515</v>
+        <v>1.7936205929235745</v>
       </c>
       <c r="L24" s="27">
-        <v>1.9474878394240012</v>
+        <v>1.7343898363661241</v>
       </c>
       <c r="M24" s="27">
-        <v>1.8084439232121547</v>
+        <v>1.5953459201542777</v>
       </c>
       <c r="N24" s="27">
-        <v>1.7657896206810266</v>
+        <v>1.5526916176231496</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.15">
@@ -12968,22 +12940,22 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="I28" s="31" t="s">
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="I28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
     </row>
     <row r="29" spans="1:14" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
@@ -13769,40 +13741,40 @@
         <v>37</v>
       </c>
       <c r="B48" s="26">
-        <v>2.5048829491088593</v>
+        <v>2.2917849460509823</v>
       </c>
       <c r="C48" s="26">
-        <v>2.5048796597928145</v>
+        <v>2.2917816567349374</v>
       </c>
       <c r="D48" s="26">
-        <v>2.5048796594239495</v>
+        <v>2.2917816563660725</v>
       </c>
       <c r="E48" s="26">
-        <v>2.5048796596087031</v>
+        <v>2.291781656550826</v>
       </c>
       <c r="F48" s="26">
-        <v>2.5048796592999794</v>
+        <v>2.2917816562421023</v>
       </c>
       <c r="G48" s="26">
-        <v>2.50487966070158</v>
+        <v>2.2917816576437029</v>
       </c>
       <c r="I48" s="27">
-        <v>2.4561042910524806</v>
+        <v>2.2430062879946036</v>
       </c>
       <c r="J48" s="27">
-        <v>2.2757499382421607</v>
+        <v>2.0626519351842836</v>
       </c>
       <c r="K48" s="27">
-        <v>2.1792973258827169</v>
+        <v>1.9661993228248398</v>
       </c>
       <c r="L48" s="27">
-        <v>2.0754465120684826</v>
+        <v>1.8623485090106056</v>
       </c>
       <c r="M48" s="27">
-        <v>1.9679381468878085</v>
+        <v>1.7548401438299315</v>
       </c>
       <c r="N48" s="27">
-        <v>1.8733675569002173</v>
+        <v>1.6602695538423402</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.15">
@@ -13845,6 +13817,51 @@
       <c r="N49" s="29">
         <v>95</v>
       </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8"/>
+      <c r="I51" s="8"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
+      <c r="L51" s="8"/>
+      <c r="M51" s="8"/>
+      <c r="N51" s="8"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="8"/>
+      <c r="J52" s="8"/>
+      <c r="K52" s="8"/>
+      <c r="L52" s="8"/>
+      <c r="M52" s="8"/>
+      <c r="N52" s="8"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="I53" s="8"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="8"/>
+      <c r="L53" s="8"/>
+      <c r="M53" s="8"/>
+      <c r="N53" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -13892,22 +13909,22 @@
     </row>
     <row r="4" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12"/>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="I4" s="31" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="I4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
     </row>
     <row r="5" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A5" s="19" t="s">
@@ -14819,40 +14836,40 @@
         <v>37</v>
       </c>
       <c r="B24" s="26">
-        <v>2.2802389000653194</v>
+        <v>2.0671408970074423</v>
       </c>
       <c r="C24" s="26">
-        <v>2.2802389037642188</v>
+        <v>2.0671409007063417</v>
       </c>
       <c r="D24" s="26">
-        <v>2.2802388933755888</v>
+        <v>2.0671408903177118</v>
       </c>
       <c r="E24" s="26">
-        <v>2.2802388883566942</v>
+        <v>2.0671408852988171</v>
       </c>
       <c r="F24" s="26">
-        <v>2.2802389124681683</v>
+        <v>2.0671409094102913</v>
       </c>
       <c r="G24" s="26">
-        <v>2.2802388806191285</v>
+        <v>2.0671408775612514</v>
       </c>
       <c r="I24" s="27">
-        <v>2.2802389000653194</v>
+        <v>2.0671408970074423</v>
       </c>
       <c r="J24" s="27">
-        <v>2.1131728546697159</v>
+        <v>1.9000748516118389</v>
       </c>
       <c r="K24" s="27">
-        <v>2.0632629087809411</v>
+        <v>1.850164905723064</v>
       </c>
       <c r="L24" s="27">
-        <v>2.0199607539238005</v>
+        <v>1.8068627508659234</v>
       </c>
       <c r="M24" s="27">
-        <v>1.972262501408218</v>
+        <v>1.7591644983503409</v>
       </c>
       <c r="N24" s="27">
-        <v>1.9205309105862522</v>
+        <v>1.7074329075283752</v>
       </c>
       <c r="Q24" s="17"/>
       <c r="R24" s="14"/>
@@ -14912,22 +14929,22 @@
     </row>
     <row r="28" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12"/>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="I28" s="31" t="s">
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="I28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
     </row>
     <row r="29" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A29" s="19" t="s">
@@ -15802,40 +15819,40 @@
         <v>37</v>
       </c>
       <c r="B48" s="26">
-        <v>2.4364032993835236</v>
+        <v>2.2233052963256466</v>
       </c>
       <c r="C48" s="26">
-        <v>2.4364042023622092</v>
+        <v>2.2233061993043322</v>
       </c>
       <c r="D48" s="26">
-        <v>2.436405565526059</v>
+        <v>2.223307562468182</v>
       </c>
       <c r="E48" s="26">
-        <v>2.4364032993834774</v>
+        <v>2.2233052963256004</v>
       </c>
       <c r="F48" s="26">
-        <v>2.4364049409405246</v>
+        <v>2.2233069378826475</v>
       </c>
       <c r="G48" s="26">
-        <v>2.4364032993834783</v>
+        <v>2.2233052963256013</v>
       </c>
       <c r="I48" s="27">
-        <v>2.4364032993835236</v>
+        <v>2.2233052963256466</v>
       </c>
       <c r="J48" s="27">
-        <v>2.3047976853435577</v>
+        <v>2.0916996822856806</v>
       </c>
       <c r="K48" s="27">
-        <v>2.2143165016950652</v>
+        <v>2.0012184986371881</v>
       </c>
       <c r="L48" s="27">
-        <v>2.0904361585545219</v>
+        <v>1.8773381554966448</v>
       </c>
       <c r="M48" s="27">
-        <v>1.9811143452073907</v>
+        <v>1.7680163421495136</v>
       </c>
       <c r="N48" s="27">
-        <v>1.9332600247338647</v>
+        <v>1.7201620216759876</v>
       </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.15">
@@ -15913,22 +15930,22 @@
     </row>
     <row r="52" spans="1:23" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="12"/>
-      <c r="B52" s="31" t="s">
+      <c r="B52" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C52" s="31"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="31"/>
-      <c r="I52" s="31" t="s">
+      <c r="C52" s="30"/>
+      <c r="D52" s="30"/>
+      <c r="E52" s="30"/>
+      <c r="F52" s="30"/>
+      <c r="G52" s="30"/>
+      <c r="I52" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="J52" s="31"/>
-      <c r="K52" s="31"/>
-      <c r="L52" s="31"/>
-      <c r="M52" s="31"/>
-      <c r="N52" s="31"/>
+      <c r="J52" s="30"/>
+      <c r="K52" s="30"/>
+      <c r="L52" s="30"/>
+      <c r="M52" s="30"/>
+      <c r="N52" s="30"/>
     </row>
     <row r="53" spans="1:23" ht="30" x14ac:dyDescent="0.15">
       <c r="A53" s="19" t="s">
@@ -16850,40 +16867,40 @@
         <v>37</v>
       </c>
       <c r="B72" s="26">
-        <v>2.5405129081006703</v>
+        <v>2.3274149050427932</v>
       </c>
       <c r="C72" s="26">
-        <v>2.5405129056630957</v>
+        <v>2.3274149026052187</v>
       </c>
       <c r="D72" s="26">
-        <v>2.5405129055202544</v>
+        <v>2.3274149024623774</v>
       </c>
       <c r="E72" s="26">
-        <v>2.5405135288128609</v>
+        <v>2.3274155257549838</v>
       </c>
       <c r="F72" s="26">
-        <v>2.5405129046769255</v>
+        <v>2.3274149016190484</v>
       </c>
       <c r="G72" s="26">
-        <v>2.5405129053616475</v>
+        <v>2.3274149023037705</v>
       </c>
       <c r="I72" s="27">
-        <v>2.5422686226907549</v>
+        <v>2.3291706196328779</v>
       </c>
       <c r="J72" s="27">
-        <v>2.4163630239205318</v>
+        <v>2.2032650208626547</v>
       </c>
       <c r="K72" s="27">
-        <v>2.3215935001600503</v>
+        <v>2.1084954971021732</v>
       </c>
       <c r="L72" s="27">
-        <v>2.2279900430022463</v>
+        <v>2.0148920399443693</v>
       </c>
       <c r="M72" s="27">
-        <v>2.1046688536984641</v>
+        <v>1.8915708506405871</v>
       </c>
       <c r="N72" s="27">
-        <v>1.9834055379495998</v>
+        <v>1.7703075348917228</v>
       </c>
       <c r="Q72" s="17"/>
       <c r="R72" s="14"/>

</xml_diff>